<commit_message>
Unify all BMC_URL tasks to relative path format
All 10 URLs now use /UI/Static/#/navigate/... format.
Runtime auto-prepends https://{bmc_ip} via _resolve_url().

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/任务模板.xlsx
+++ b/examples/任务模板.xlsx
@@ -545,14 +545,11 @@
           <t>L1-示例-01</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>10.0.2.101</t>
@@ -585,14 +582,11 @@
           <t>L2-示例-01</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>10.0.3.101</t>
@@ -645,9 +639,6 @@
           <t>Admin@123</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>RM211,机柜</t>
@@ -775,7 +766,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>BMC_URL</t>
@@ -783,10 +773,9 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://{带外管理IP}/UI/Static/#/navigate/system/storage</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
+          <t>/UI/Static/#/navigate/system/storage</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -808,7 +797,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -829,7 +817,6 @@
           <t>RM211</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>BMC_URL</t>
@@ -837,10 +824,9 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://{带外管理IP}/UI/Static/#/navigate/manager/network</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
+          <t>/UI/Static/#/navigate/manager/network</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -862,7 +848,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -883,7 +868,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>BMC_URL</t>
@@ -891,10 +875,9 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://{带外管理IP}/UI/Static/#/navigate/system/power/control</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
+          <t>/UI/Static/#/navigate/system/power/control</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -916,7 +899,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -937,7 +919,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>BMC_URL</t>
@@ -948,7 +929,6 @@
           <t>/UI/Static/#/navigate/system/info/product</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -970,7 +950,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -991,7 +970,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>BMC_URL</t>
@@ -1002,7 +980,6 @@
           <t>/UI/Static/#/navigate/system/info/net</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1024,7 +1001,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1045,7 +1021,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>BMC_URL</t>
@@ -1056,7 +1031,6 @@
           <t>/UI/Static/#/navigate/system/info/sensor</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1078,7 +1052,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1099,7 +1072,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>BMC_URL</t>
@@ -1110,7 +1082,6 @@
           <t>/UI/Static/#/navigate/system/power/converter</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1132,7 +1103,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1153,7 +1123,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>BMC_URL</t>
@@ -1164,7 +1133,6 @@
           <t>/UI/Static/#/navigate/system/fans/fans-info</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1186,7 +1154,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1207,7 +1174,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>BMC_URL</t>
@@ -1218,7 +1184,6 @@
           <t>/UI/Static/#/navigate/system/power/converter</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1240,7 +1205,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1261,7 +1225,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>BMC_URL</t>
@@ -1269,10 +1232,9 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://{带外管理IP}/UI/Static/#/navigate/home</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
+          <t>/UI/Static/#/navigate/home</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1294,7 +1256,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1315,7 +1276,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>SSH_CMD</t>
@@ -1326,7 +1286,6 @@
           <t>uname -a</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1348,7 +1307,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1369,7 +1327,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>SSH_CMD</t>
@@ -1381,7 +1338,6 @@
 /usr/local/Ascend/driver/tools/upgrade-tool --device_index -1 --component -1 --version</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1403,7 +1359,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1424,7 +1379,6 @@
           <t>L1/L2</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>SSH_CMD</t>
@@ -1437,7 +1391,6 @@
 display this</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1459,7 +1412,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1480,7 +1432,6 @@
           <t>L1/L2</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>SSH_CMD</t>
@@ -1491,7 +1442,6 @@
           <t>display device elabel</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1513,7 +1463,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1534,7 +1483,6 @@
           <t>L1/L2</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>SSH_CMD</t>
@@ -1546,7 +1494,6 @@
 display version</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1568,7 +1515,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1589,7 +1535,6 @@
           <t>L1/L2</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>SSH_CMD</t>
@@ -1602,7 +1547,6 @@
 display interface 200GHL1/2/48</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1624,7 +1568,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1645,7 +1588,6 @@
           <t>L1/L2</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>SSH_CMD</t>
@@ -1656,7 +1598,6 @@
           <t>display interface transceiver</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1678,7 +1619,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1699,7 +1639,6 @@
           <t>L1/L2</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>SSH_CMD</t>
@@ -1710,7 +1649,6 @@
           <t>display device temperature</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1732,7 +1670,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1753,7 +1690,6 @@
           <t>L1</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>SSH_CMD</t>
@@ -1764,7 +1700,6 @@
           <t>display interface brief | include up</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1786,7 +1721,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1807,7 +1741,6 @@
           <t>L1/L2</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>SSH_CMD</t>
@@ -1818,7 +1751,6 @@
           <t>display interface brief</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1840,7 +1772,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1861,13 +1792,11 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>CUSTOM_SCRIPT</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>BMC 上电测试-内存证据采集</t>
@@ -1894,7 +1823,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1915,13 +1843,11 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>CUSTOM_SCRIPT</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>BMC 上电测试-CPU 证据采集</t>
@@ -1948,7 +1874,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1969,13 +1894,11 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>CUSTOM_SCRIPT</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>iBMC IP/网络设置类证据</t>
@@ -2002,7 +1925,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2023,13 +1945,11 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>CUSTOM_SCRIPT</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>CPU 部件信息采集</t>
@@ -2056,7 +1976,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2077,13 +1996,11 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>CUSTOM_SCRIPT</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>NPU 部件信息采集</t>
@@ -2110,7 +2027,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2131,13 +2047,11 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>CUSTOM_SCRIPT</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>内存部件信息采集</t>
@@ -2164,7 +2078,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2185,13 +2098,11 @@
           <t>RM211</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>CUSTOM_SCRIPT</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>RM211 电源冗余/系统事件证据</t>
@@ -2218,7 +2129,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2239,13 +2149,11 @@
           <t>RM211</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>CUSTOM_SCRIPT</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>系统日志证据</t>
@@ -2272,7 +2180,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2293,13 +2200,11 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>CUSTOM_SCRIPT</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>A3 硬盘冗余/logical drive 证据</t>
@@ -2326,7 +2231,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2347,13 +2251,11 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>CUSTOM_SCRIPT</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>ClearForeign 配置类高风险任务</t>
@@ -2380,7 +2282,6 @@
           <t>否</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Split task config: Excel (matching) + tasks.json (execution details)
- tasks.json: 30 task definitions with URLs/commands/timeouts/rules
- Excel simplified to 8 columns: seq/name/type/group/tags/outdir/imgname/enabled
- Loader merges by task name — JSON priority, Excel fallback
- CUSTOM_SCRIPT tasks auto-disabled unless explicitly enabled in JSON
- Agent can push updated tasks.json without touching Excel

Also fix Windows robocopy exit code handling in CI/CD.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/任务模板.xlsx
+++ b/examples/任务模板.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="设备信息" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="任务列表" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="任务分类说明" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="说明" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -545,11 +545,14 @@
           <t>L1-示例-01</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>10.0.2.101</t>
@@ -582,11 +585,14 @@
           <t>L2-示例-01</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>10.0.3.101</t>
@@ -639,6 +645,9 @@
           <t>Admin@123</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>RM211,机柜</t>
@@ -656,7 +665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -664,15 +673,9 @@
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="42" customWidth="1" min="9" max="9"/>
-    <col width="42" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -703,47 +706,17 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>执行模式</t>
+          <t>截图保存目录</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>执行命令/URL</t>
+          <t>图片命名格式</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Actions JSON/规则JSON</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>截图保存目录</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>图片命名格式</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>超时时间(秒)</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>重试次数</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
           <t>是否启用</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>规则JSON</t>
         </is>
       </c>
     </row>
@@ -766,33 +739,18 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>BMC_URL</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>/UI/Static/#/navigate/system/storage</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>60</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="inlineStr">
+          <t>{device_name}_{task_name}_{timestamp}</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -817,33 +775,18 @@
           <t>RM211</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>BMC_URL</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>/UI/Static/#/navigate/manager/network</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K3" t="n">
-        <v>60</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" t="inlineStr">
+          <t>{device_name}_{task_name}_{timestamp}</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -868,33 +811,18 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>BMC_URL</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>/UI/Static/#/navigate/system/power/control</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>60</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" t="inlineStr">
+          <t>{device_name}_{task_name}_{timestamp}</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -919,33 +847,18 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>BMC_URL</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>/UI/Static/#/navigate/system/info/product</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>60</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" t="inlineStr">
+          <t>{device_name}_{task_name}_{timestamp}</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -970,33 +883,18 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>BMC_URL</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>/UI/Static/#/navigate/system/info/net</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
-        <v>60</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="inlineStr">
+          <t>{device_name}_{task_name}_{timestamp}</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1021,33 +919,18 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>BMC_URL</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>/UI/Static/#/navigate/system/info/sensor</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K7" t="n">
-        <v>60</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" t="inlineStr">
+          <t>{device_name}_{task_name}_{timestamp}</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1072,33 +955,18 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>BMC_URL</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>/UI/Static/#/navigate/system/power/converter</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K8" t="n">
-        <v>60</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" t="inlineStr">
+          <t>{device_name}_{task_name}_{timestamp}</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1123,33 +991,18 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>BMC_URL</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>/UI/Static/#/navigate/system/fans/fans-info</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K9" t="n">
-        <v>60</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" t="inlineStr">
+          <t>{device_name}_{task_name}_{timestamp}</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1174,33 +1027,18 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>BMC_URL</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>/UI/Static/#/navigate/system/power/converter</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K10" t="n">
-        <v>60</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" t="inlineStr">
+          <t>{device_name}_{task_name}_{timestamp}</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1225,33 +1063,18 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>BMC_URL</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>/UI/Static/#/navigate/home</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K11" t="n">
-        <v>60</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" t="inlineStr">
+          <t>{device_name}_{task_name}_{timestamp}</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1276,33 +1099,18 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>SSH_CMD</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>uname -a</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K12" t="n">
-        <v>60</v>
-      </c>
-      <c r="L12" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" t="inlineStr">
+          <t>{device_name}_{task_name}_{timestamp}</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1327,34 +1135,18 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>SSH_CMD</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>npu-smi info
-/usr/local/Ascend/driver/tools/upgrade-tool --device_index -1 --component -1 --version</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K13" t="n">
-        <v>60</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" t="inlineStr">
+          <t>{device_name}_{task_name}_{timestamp}</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1379,35 +1171,18 @@
           <t>L1/L2</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>SSH_CMD</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>system-view
-interface MEth0/0/0
-display this</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K14" t="n">
-        <v>60</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" t="inlineStr">
+          <t>{device_name}_{task_name}_{timestamp}</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1432,33 +1207,18 @@
           <t>L1/L2</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>SSH_CMD</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>display device elabel</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K15" t="n">
-        <v>60</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" t="inlineStr">
+          <t>{device_name}_{task_name}_{timestamp}</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1483,34 +1243,18 @@
           <t>L1/L2</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>SSH_CMD</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>display device card
-display version</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K16" t="n">
-        <v>60</v>
-      </c>
-      <c r="L16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" t="inlineStr">
+          <t>{device_name}_{task_name}_{timestamp}</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1535,35 +1279,18 @@
           <t>L1/L2</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>SSH_CMD</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>screen-length 0 temporary
-display interface brief
-display interface 200GHL1/2/48</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K17" t="n">
-        <v>60</v>
-      </c>
-      <c r="L17" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" t="inlineStr">
+          <t>{device_name}_{task_name}_{timestamp}</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1588,33 +1315,18 @@
           <t>L1/L2</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>SSH_CMD</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>display interface transceiver</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K18" t="n">
-        <v>60</v>
-      </c>
-      <c r="L18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" t="inlineStr">
+          <t>{device_name}_{task_name}_{timestamp}</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1639,33 +1351,18 @@
           <t>L1/L2</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>SSH_CMD</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>display device temperature</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K19" t="n">
-        <v>60</v>
-      </c>
-      <c r="L19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" t="inlineStr">
+          <t>{device_name}_{task_name}_{timestamp}</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1690,33 +1387,18 @@
           <t>L1</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>SSH_CMD</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>display interface brief | include up</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K20" t="n">
-        <v>60</v>
-      </c>
-      <c r="L20" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" t="inlineStr">
+          <t>{device_name}_{task_name}_{timestamp}</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1741,33 +1423,18 @@
           <t>L1/L2</t>
         </is>
       </c>
+      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>SSH_CMD</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>display interface brief</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K21" t="n">
-        <v>60</v>
-      </c>
-      <c r="L21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" t="inlineStr">
+          <t>{device_name}_{task_name}_{timestamp}</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1792,33 +1459,18 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>CUSTOM_SCRIPT</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
-        <is>
-          <t>BMC 上电测试-内存证据采集</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K22" t="n">
-        <v>120</v>
-      </c>
-      <c r="L22" t="n">
-        <v>0</v>
-      </c>
-      <c r="M22" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -1843,33 +1495,18 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
-          <t>CUSTOM_SCRIPT</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
-        <is>
-          <t>BMC 上电测试-CPU 证据采集</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K23" t="n">
-        <v>120</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -1894,33 +1531,18 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
-          <t>CUSTOM_SCRIPT</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
-        <is>
-          <t>iBMC IP/网络设置类证据</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K24" t="n">
-        <v>120</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -1945,33 +1567,18 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>CUSTOM_SCRIPT</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
-        <is>
-          <t>CPU 部件信息采集</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K25" t="n">
-        <v>120</v>
-      </c>
-      <c r="L25" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -1996,33 +1603,18 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
-          <t>CUSTOM_SCRIPT</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
-        <is>
-          <t>NPU 部件信息采集</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K26" t="n">
-        <v>120</v>
-      </c>
-      <c r="L26" t="n">
-        <v>0</v>
-      </c>
-      <c r="M26" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -2047,33 +1639,18 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
-          <t>CUSTOM_SCRIPT</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
-        <is>
-          <t>内存部件信息采集</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K27" t="n">
-        <v>120</v>
-      </c>
-      <c r="L27" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -2098,33 +1675,18 @@
           <t>RM211</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>CUSTOM_SCRIPT</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
-        <is>
-          <t>RM211 电源冗余/系统事件证据</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K28" t="n">
-        <v>120</v>
-      </c>
-      <c r="L28" t="n">
-        <v>0</v>
-      </c>
-      <c r="M28" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -2149,33 +1711,18 @@
           <t>RM211</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
-          <t>CUSTOM_SCRIPT</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
-        <is>
-          <t>系统日志证据</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K29" t="n">
-        <v>120</v>
-      </c>
-      <c r="L29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M29" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -2200,33 +1747,18 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
-          <t>CUSTOM_SCRIPT</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
-        <is>
-          <t>A3 硬盘冗余/logical drive 证据</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K30" t="n">
-        <v>120</v>
-      </c>
-      <c r="L30" t="n">
-        <v>0</v>
-      </c>
-      <c r="M30" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -2238,7 +1770,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>拔插硬盘后清除Foreign配置 (高风险-必须禁用)</t>
+          <t>拔插硬盘后清除Foreign配置</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2251,33 +1783,18 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
-          <t>CUSTOM_SCRIPT</t>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
-        <is>
-          <t>ClearForeign 配置类高风险任务</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="K31" t="n">
-        <v>120</v>
-      </c>
-      <c r="L31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M31" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -2294,193 +1811,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>执行模式</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>数量</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>说明</t>
+          <t>任务配置分为两层：</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BMC_URL</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>登录 BMC 后打开指定 URL，截图 + 保存 HTML。URL 支持模板变量 {带外管理IP}</t>
+          <t>1. Excel 任务列表 — 只配置匹配信息：序号/名称/类型/分组/标签/输出目录/命名格式/启用</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SSH_CMD</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>SSH 登录带内 IP，执行命令，保存 TXT 输出。多命令用换行分隔</t>
+          <t>2. tasks.json — 执行细节：URL/命令/超时/重试/规则，通过任务名称匹配</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CUSTOM_SCRIPT</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>遗留复杂脚本，已全部禁用。后续用 BMC_ACTIONS + 规则体系替代</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>BMC_ACTIONS</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>DSL 复杂 BMC 操作。支持 goto/click/fill/screenshot/assert/wait 等动作，JSON 格式配置</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>设备分组</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>旧版设备数</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>主要任务类型</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>A3</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>96</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>BMC_URL + SSH_CMD(uname/npu)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>L1</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>96</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>SSH_CMD(display 命令)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>L2</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>112</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>SSH_CMD(display 命令)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>RM211</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>64</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>BMC_URL(机柜管理)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>注意</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>CUSTOM_SCRIPT 遗留任务需要逐个评估，将可迁移的转为 BMC_ACTIONS 或规则，不可迁移的保持禁用</t>
+          <t>Agent 可远程推送更新 tasks.json，无需修改 Excel</t>
         </is>
       </c>
     </row>

</xml_diff>